<commit_message>
feat(itrust-study): publish specification and test suite v8.0
</commit_message>
<xml_diff>
--- a/output/xlsx/UC14AlertUsersByEmail--GT-.xlsx
+++ b/output/xlsx/UC14AlertUsersByEmail--GT-.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="37">
   <si>
     <t xml:space="preserve">System: </t>
   </si>
@@ -29,7 +29,7 @@
     <t xml:space="preserve">Version: </t>
   </si>
   <si>
-    <t>7.0</t>
+    <t>8.0</t>
   </si>
   <si>
     <t>Suite Type:</t>
@@ -38,7 +38,7 @@
     <t>Reduced (Greedy Heuristic - Transition Coverage)</t>
   </si>
   <si>
-    <t>Size: 4 test case(s)</t>
+    <t>Size: 3 test case(s)</t>
   </si>
   <si>
     <t xml:space="preserve">Creation Date: </t>
@@ -123,18 +123,6 @@
   </si>
   <si>
     <t>user: A user account has been locked out, either temporarily or permanently, due to too many failed logins. An email informing the user of their lockout is sent.</t>
-  </si>
-  <si>
-    <t>TC4</t>
-  </si>
-  <si>
-    <t>Exception Flow 1: No valid email associated with account</t>
-  </si>
-  <si>
-    <t>SYSTEM prompts that If the user does not have an email address on file, no email is sent and the failure is logged.</t>
-  </si>
-  <si>
-    <t>Flow interrupted due to exception / error</t>
   </si>
 </sst>
 </file>
@@ -226,13 +214,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="148.84765625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="21.8984375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="91.7109375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="45.98828125" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="30.5234375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="17.578125" customWidth="true" bestFit="true"/>
   </cols>
@@ -519,87 +507,6 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B30" t="s" s="0">
-        <v>37</v>
-      </c>
-      <c r="C30" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E30" t="s" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="B31" t="s" s="0">
-        <v>38</v>
-      </c>
-      <c r="E31" t="s" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="B32" t="s" s="0">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="B33" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="C33" t="s" s="2">
-        <v>22</v>
-      </c>
-      <c r="D33" t="s" s="2">
-        <v>23</v>
-      </c>
-      <c r="E33" t="s" s="2">
-        <v>24</v>
-      </c>
-      <c r="F33" t="s" s="2">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B34" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C34" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D34" t="s" s="3">
-        <v>39</v>
-      </c>
-      <c r="E34" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F34" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="s" s="1">
-        <v>29</v>
-      </c>
-      <c r="B35" t="s" s="0">
-        <v>40</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>